<commit_message>
Add Nuclear + GDP PPP to observed data (6 variables)
</commit_message>
<xml_diff>
--- a/data/observed.xlsx
+++ b/data/observed.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,16 @@
           <t>source</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -477,6 +487,12 @@
           <t>GCB 2025</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -500,6 +516,12 @@
           <t>GCB 2025</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -523,6 +545,16 @@
           <t>GCB 2025</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>COVID dip</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -546,6 +578,16 @@
           <t>GCB 2025</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>GCB=38.1Gt IEA=38.4Gt</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -569,6 +611,16 @@
           <t>EI StatReview 2025</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -592,6 +644,16 @@
           <t>EI StatReview 2025</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -615,6 +677,16 @@
           <t>EI StatReview 2025</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>COVID dip</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -638,6 +710,16 @@
           <t>EI StatReview 2025</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>record high</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -661,6 +743,12 @@
           <t>IRENA 2026</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -684,6 +772,12 @@
           <t>IRENA 2026</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -707,6 +801,12 @@
           <t>IRENA 2026</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -730,6 +830,12 @@
           <t>IRENA 2026</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -753,6 +859,12 @@
           <t>IRENA 2026</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -776,6 +888,12 @@
           <t>IRENA 2026</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -799,6 +917,12 @@
           <t>IRENA 2026</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -820,6 +944,268 @@
       <c r="E17" t="inlineStr">
         <is>
           <t>IRENA 2026</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Capacity|Electricity|Nuclear</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C18" t="n">
+        <v>375</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>IAEA PRIS</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>pre-Fukushima</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Capacity|Electricity|Nuclear</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C19" t="n">
+        <v>383</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>IAEA PRIS</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>post-Fukushima recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Capacity|Electricity|Nuclear</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C20" t="n">
+        <v>393</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>IAEA PRIS</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>operable capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Capacity|Electricity|Nuclear</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C21" t="n">
+        <v>377</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>IAEA PRIS</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>IAEA end-2024: 377 GW(e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GDP|PPP</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C22" t="n">
+        <v>87774</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>billion US$2010/yr</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>IMF WEO / World Bank</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GDP|PPP</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C23" t="n">
+        <v>100690</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>billion US$2010/yr</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>IMF WEO / World Bank</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GDP|PPP</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C24" t="n">
+        <v>107100</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>billion US$2010/yr</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>IMF WEO / World Bank</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>COVID dip</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GDP|PPP</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C25" t="n">
+        <v>122000</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>billion US$2010/yr</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>IMF WEO / World Bank</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>CHECK UNIT: SCI may use US$2005 not US$2010</t>
         </is>
       </c>
     </row>

</xml_diff>